<commit_message>
chore: update HEBREW_Sessions_Communications.xlsx with corrected version
</commit_message>
<xml_diff>
--- a/HEBREW_Sessions_Communications.xlsx
+++ b/HEBREW_Sessions_Communications.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ariel\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4FBA43E-1ADB-4C73-A68C-DAC4D958D8E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36EF01D9-E7C8-4BC9-946C-E2F17BE4EEBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BFF36C6D-0428-4B5F-A930-B6FB065C0601}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{BFF36C6D-0428-4B5F-A930-B6FB065C0601}"/>
   </bookViews>
   <sheets>
     <sheet name="Automation" sheetId="1" r:id="rId1"/>
     <sheet name="Communication" sheetId="2" r:id="rId2"/>
+    <sheet name="Examples" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="70">
   <si>
     <t>מצב</t>
   </si>
@@ -303,12 +304,63 @@
   <si>
     <t>מה נטען (נשלח ל-AI)</t>
   </si>
+  <si>
+    <t>כל שעה יתריע כושר</t>
+  </si>
+  <si>
+    <t>אם פספסתי פעמיים אז לא להתריע</t>
+  </si>
+  <si>
+    <t>אם דיווחתי להתניע מחדש</t>
+  </si>
+  <si>
+    <t>ותמיד בצורה משעשעת</t>
+  </si>
+  <si>
+    <t>delivery</t>
+  </si>
+  <si>
+    <t>דוגמת אבטחה</t>
+  </si>
+  <si>
+    <t>דוגמת אריאל</t>
+  </si>
+  <si>
+    <t>כל יום סקירת אבטחה</t>
+  </si>
+  <si>
+    <t>אם יש סוגייה, תטפל בה</t>
+  </si>
+  <si>
+    <t>אם היה טיפול, תעדכן אותי</t>
+  </si>
+  <si>
+    <t>כלי?</t>
+  </si>
+  <si>
+    <t>cron isolated</t>
+  </si>
+  <si>
+    <t>מסקנה ל session_send</t>
+  </si>
+  <si>
+    <t>session_send</t>
+  </si>
+  <si>
+    <t>אחרת תתריע</t>
+  </si>
+  <si>
+    <t>DB</t>
+  </si>
+  <si>
+    <t>NEW</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -354,8 +406,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -430,6 +503,21 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -568,7 +656,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="11">
+  <cellStyleXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -580,8 +668,11 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -655,12 +746,60 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="8" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="10" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="8" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="3" xfId="10" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="10" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="3" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -670,62 +809,21 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="5" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="2" xfId="9" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="10" xfId="10" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="8" xfId="10" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="3" xfId="10" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="10" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="3" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="10" xfId="8" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="3" xfId="8" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="2" xfId="13" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="2" xfId="12" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="2" xfId="11" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="11">
+  <cellStyles count="14">
     <cellStyle name="20% - Accent6" xfId="10" builtinId="50"/>
     <cellStyle name="40% - Accent4" xfId="9" builtinId="43"/>
     <cellStyle name="60% - Accent4" xfId="5" builtinId="44"/>
@@ -735,7 +833,10 @@
     <cellStyle name="Accent3" xfId="3" builtinId="37"/>
     <cellStyle name="Accent4" xfId="4" builtinId="41"/>
     <cellStyle name="Accent5" xfId="6" builtinId="45"/>
+    <cellStyle name="Bad" xfId="12" builtinId="27"/>
+    <cellStyle name="Good" xfId="11" builtinId="26"/>
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
+    <cellStyle name="Neutral" xfId="13" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1123,7 +1224,7 @@
       <c r="H4" s="13"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="32" t="s">
         <v>4</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1146,7 +1247,7 @@
       </c>
     </row>
     <row r="6" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B6" s="25"/>
+      <c r="B6" s="32"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -1155,8 +1256,8 @@
       <c r="H6" s="1"/>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B7" s="25"/>
-      <c r="C7" s="46" t="s">
+      <c r="B7" s="32"/>
+      <c r="C7" s="30" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -1185,7 +1286,7 @@
       <c r="H8" s="1"/>
     </row>
     <row r="9" spans="2:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="33" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="19" t="s">
@@ -1208,7 +1309,7 @@
       </c>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B10" s="26"/>
+      <c r="B10" s="33"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -1217,8 +1318,8 @@
       <c r="H10" s="1"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B11" s="26"/>
-      <c r="C11" s="47" t="s">
+      <c r="B11" s="33"/>
+      <c r="C11" s="31" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="6" t="s">
@@ -1238,7 +1339,7 @@
       </c>
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="26"/>
+      <c r="B12" s="33"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -1246,7 +1347,7 @@
       <c r="H12" s="1"/>
     </row>
     <row r="13" spans="2:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="B13" s="26"/>
+      <c r="B13" s="33"/>
       <c r="C13" s="20" t="s">
         <v>22</v>
       </c>
@@ -1344,7 +1445,7 @@
       <c r="E5" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="27" t="s">
+      <c r="F5" s="43" t="s">
         <v>16</v>
       </c>
     </row>
@@ -1355,45 +1456,45 @@
       <c r="C6" s="40"/>
       <c r="D6" s="40"/>
       <c r="E6" s="42"/>
-      <c r="F6" s="28"/>
+      <c r="F6" s="44"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="C8" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="D8" s="31"/>
+      <c r="D8" s="26"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="32"/>
+      <c r="D9" s="27"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B10" s="30" t="s">
+      <c r="B10" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="33"/>
+      <c r="D10" s="28"/>
     </row>
     <row r="12" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="29" t="s">
+      <c r="C12" s="45" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
+      <c r="D12" s="45"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="45"/>
       <c r="G12" s="24" t="s">
         <v>44</v>
       </c>
@@ -1402,60 +1503,60 @@
       <c r="B13" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="44" t="s">
+      <c r="C13" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
+      <c r="D13" s="35"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="35"/>
       <c r="G13" s="36" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B14" s="43" t="s">
+      <c r="B14" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="44" t="s">
+      <c r="C14" s="34" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
       <c r="G14" s="37"/>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="C15" s="45" t="s">
+      <c r="C15" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="35"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
+      <c r="D15" s="47"/>
+      <c r="E15" s="47"/>
+      <c r="F15" s="47"/>
       <c r="G15" s="37"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
       <c r="G16" s="37"/>
     </row>
     <row r="17" spans="2:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C17" s="44" t="s">
+      <c r="C17" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="D17" s="34"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="34"/>
+      <c r="D17" s="35"/>
+      <c r="E17" s="35"/>
+      <c r="F17" s="35"/>
       <c r="G17" s="38"/>
     </row>
   </sheetData>
@@ -1473,4 +1574,130 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D3050BD-FA2F-44E0-8E38-D51A4385130F}">
+  <dimension ref="B2:H9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="30" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.28515625" customWidth="1"/>
+    <col min="7" max="7" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="51" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="F3" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" s="49"/>
+      <c r="H3" s="49" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B5" s="48">
+        <v>1</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="50" t="s">
+        <v>64</v>
+      </c>
+      <c r="F5" s="48">
+        <v>1</v>
+      </c>
+      <c r="G5" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" s="50" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B6" s="48">
+        <v>1.5</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="48" t="s">
+        <v>66</v>
+      </c>
+      <c r="F6" s="48">
+        <v>2</v>
+      </c>
+      <c r="G6" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="H6" s="50" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B7" s="48">
+        <v>2</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="48" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="48">
+        <v>3</v>
+      </c>
+      <c r="G7" s="48" t="s">
+        <v>62</v>
+      </c>
+      <c r="H7" s="48" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="48">
+        <v>3</v>
+      </c>
+      <c r="C8" s="48" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="51" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="48">
+        <v>4</v>
+      </c>
+      <c r="C9" s="48" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="52" t="s">
+        <v>69</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>